<commit_message>
UX: remove unnecessary Enter prompts (step1→2, step2→3, auto-prep→menu, option4 end) + merge duplicate y/n in option5
</commit_message>
<xml_diff>
--- a/uctalent_jobs.xlsx
+++ b/uctalent_jobs.xlsx
@@ -704,12 +704,8 @@
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>Hi [FirstName],
-I came across your profile and was impressed by your background. We're helping a client fill a Fraud &amp; Risk Specialist/Leader role based in Hanoi, Vietnam (₫30,000,000-₫35,000,000/monthly), and your experience seems like a strong match.
-The role focuses on: Human Resource (HR), Software and IT Services, Team Management.
-Would you be open to a quick chat to explore this opportunity?
-Best regards,
-Nhat - UCTalent</t>
+          <t>Hi [Name], impressed by your risk management and data analysis background. I'm recruiting a Fraud &amp; Risk Specialist/Leader in Hanoi (₫30-35M/month) for a client — strong fit for your KYC, SQL, and leadership experience. Open to a brief chat?
+Best regards</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr"/>
@@ -727,7 +723,7 @@
       </c>
       <c r="W2" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>ready_to_connect</t>
         </is>
       </c>
       <c r="X2" s="2" t="inlineStr">
@@ -2494,7 +2490,7 @@
       </c>
       <c r="U15" s="3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/stevendu,https://www.linkedin.com/in/aloysius-ekezie-65419224b,https://www.linkedin.com/in/amen-stoney-214452230,https://www.linkedin.com/in/dmitriy-polumiskov,https://www.linkedin.com/in/alexei-rusu-dev,https://linkedin.com/in/nicholas-ericksen-993b66ab,https://www.linkedin.com/in/moelh,https://www.linkedin.com/in/joel-francis-541821305,https://www.linkedin.com/in/timambler,https://www.linkedin.com/in/crystalcardona,https://www.linkedin.com/in/adeel-bukhari-4521635,https://www.linkedin.com/in/ameinalmoughrabi,https://www.linkedin.com/in/daniel-ho7,https://www.linkedin.com/in/chrisjagius,https://www.linkedin.com/in/ilan-rouson-b8aa5562,https://www.linkedin.com/in/contreras9,https://www.linkedin.com/in/mohammed-bensassi,https://www.linkedin.com/in/mohamed-elmahy</t>
+          <t>https://www.linkedin.com/in/stevendu,https://www.linkedin.com/in/aloysius-ekezie-65419224b,https://www.linkedin.com/in/amen-stoney-214452230,https://www.linkedin.com/in/dmitriy-polumiskov,https://www.linkedin.com/in/alexei-rusu-dev,https://linkedin.com/in/nicholas-ericksen-993b66ab,https://www.linkedin.com/in/moelh,https://www.linkedin.com/in/joel-francis-541821305,https://www.linkedin.com/in/timambler,https://www.linkedin.com/in/crystalcardona,https://www.linkedin.com/in/adeel-bukhari-4521635,https://www.linkedin.com/in/ameinalmoughrabi,https://www.linkedin.com/in/daniel-ho7,https://www.linkedin.com/in/chrisjagius,https://www.linkedin.com/in/ilan-rouson-b8aa5562,https://www.linkedin.com/in/contreras9,https://www.linkedin.com/in/mohammed-bensassi,https://www.linkedin.com/in/mohamed-elmahy,https://www.linkedin.com/in/anton-james-ja,https://www.linkedin.com/in/navdeepkumar2025,https://www.linkedin.com/in/oswaldo-almazo</t>
         </is>
       </c>
       <c r="V15" s="2" t="inlineStr">
@@ -2536,7 +2532,7 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>https://uctalent.io/referral/BirthdayN/truVABkpOttB6r2_Fm7J4?utm_source=headhunter&amp;utm_medium=referral</t>
+          <t>https://uctalent.io/referral/BirthdayN/qYg0VbSBL3DcpYkSBXeQK?utm_source=headhunter&amp;utm_medium=referral</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -2586,12 +2582,8 @@
       </c>
       <c r="M16" s="3" t="inlineStr">
         <is>
-          <t>Hi [FirstName],
-I came across your profile and was impressed by your experience. We're currently hiring for a Software Engineer role based in New York, United States ($150,000-$215,000/annually), and your background seems like a great match.
-Key skills we're looking for: Engineering, Software and IT Services, Node.js.
-Would you be open to a quick chat to explore this opportunity?
-Best regards,
-Nhat - UCTalent</t>
+          <t>Hi — your background in Node.js, React, and AWS infrastructure caught my attention. I'm representing a client in New York hiring a Software Engineer ($150K–$215K) with your stack. Worth a quick chat if you're open to it?
+Best regards</t>
         </is>
       </c>
       <c r="N16" s="3" t="inlineStr">
@@ -2660,7 +2652,11 @@
 https://uctalent.io/referral/BirthdayN/truVABkpOttB6r2Fm7J4?utmsource=headhunter&amp;utm_medium=referral</t>
         </is>
       </c>
-      <c r="U16" s="3" t="inlineStr"/>
+      <c r="U16" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/stevendu,https://www.linkedin.com/in/aloysius-ekezie-65419224b,https://www.linkedin.com/in/amen-stoney-214452230,https://www.linkedin.com/in/dmitriy-polumiskov,https://www.linkedin.com/in/alexei-rusu-dev,https://linkedin.com/in/nicholas-ericksen-993b66ab,https://www.linkedin.com/in/moelh,https://www.linkedin.com/in/joel-francis-541821305,https://www.linkedin.com/in/timambler,https://www.linkedin.com/in/crystalcardona,https://www.linkedin.com/in/anton-james-ja,https://www.linkedin.com/in/adeel-bukhari-4521635,https://www.linkedin.com/in/ameinalmoughrabi,https://www.linkedin.com/in/daniel-ho7,https://www.linkedin.com/in/chrisjagius,https://www.linkedin.com/in/ilan-rouson-b8aa5562,https://www.linkedin.com/in/mohammed-bensassi,https://www.linkedin.com/in/contreras9,https://www.linkedin.com/in/navdeepkumar2025,https://www.linkedin.com/in/oswaldo-almazo</t>
+        </is>
+      </c>
       <c r="V16" s="2" t="inlineStr">
         <is>
           <t>pending</t>
@@ -2668,7 +2664,7 @@
       </c>
       <c r="W16" s="2" t="inlineStr">
         <is>
-          <t>searching</t>
+          <t>ready_to_connect</t>
         </is>
       </c>
       <c r="X16" s="2" t="inlineStr">

</xml_diff>